<commit_message>
Edite scraper_flashscore.py para extraer varias ligas y copas. A su vez extraigo nuevas variables: probabilidades de bet365, lista de jugadores titulares y suplentees
Extraigo nuevas entidades como (jugador o atrib_jug) puesto que implemente la idea de usar varios datasets e integrarlos todos en uno solo (especificamente, en el de entidad partido).

Desarrolle scraper_sofifa.py para obtener datos de jugadores. Extraje los jugadores de todas las ligas de sudamerica

Desarrolle entidad atrib_jugadores para tener los datos de cada jugador en cada año.
</commit_message>
<xml_diff>
--- a/data_understanding/collect_data/entidad_competicion.xlsx
+++ b/data_understanding/collect_data/entidad_competicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07039F26-2DFD-E140-B0A3-3490E561ABDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5F652D-8B94-A448-83B9-765DC03EF019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -80,9 +80,6 @@
     <t>Bolivia</t>
   </si>
   <si>
-    <t>División Profesional</t>
-  </si>
-  <si>
     <t>Liga</t>
   </si>
   <si>
@@ -146,9 +143,6 @@
     <t>Copa Bicentenario</t>
   </si>
   <si>
-    <t>Copa Perú</t>
-  </si>
-  <si>
     <t>Supercopa Peruana</t>
   </si>
   <si>
@@ -180,6 +174,12 @@
   </si>
   <si>
     <t>Sudamerica</t>
+  </si>
+  <si>
+    <t>Division Profesional</t>
+  </si>
+  <si>
+    <t>Copa Peru</t>
   </si>
 </sst>
 </file>
@@ -565,7 +565,7 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
         <v>4</v>
@@ -580,7 +580,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
         <v>4</v>
@@ -595,7 +595,7 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
         <v>4</v>
@@ -610,7 +610,7 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
@@ -625,7 +625,7 @@
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
         <v>4</v>
@@ -640,7 +640,7 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D7" t="s">
         <v>4</v>
@@ -655,7 +655,7 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
         <v>4</v>
@@ -667,10 +667,10 @@
         <v>8DivBol</v>
       </c>
       <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" t="s">
         <v>14</v>
-      </c>
-      <c r="C9" t="s">
-        <v>15</v>
       </c>
       <c r="D9" t="s">
         <v>13</v>
@@ -682,10 +682,10 @@
         <v>9LeaBol</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D10" t="s">
         <v>13</v>
@@ -697,13 +697,13 @@
         <v>10BraBra</v>
       </c>
       <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" t="s">
         <v>18</v>
-      </c>
-      <c r="C11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D11" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -712,13 +712,13 @@
         <v>11CopBra</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -727,13 +727,13 @@
         <v>12SupBra</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -742,10 +742,10 @@
         <v>13PriChi</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
@@ -757,10 +757,10 @@
         <v>14CopChi</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -775,7 +775,7 @@
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
@@ -787,13 +787,13 @@
         <v>16PriCol</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -802,13 +802,13 @@
         <v>17CopCol</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -817,13 +817,13 @@
         <v>18SupCol</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -832,13 +832,13 @@
         <v>19LigEcu</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -847,13 +847,13 @@
         <v>20CopEcu</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -865,10 +865,10 @@
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -877,13 +877,13 @@
         <v>22PriPar</v>
       </c>
       <c r="B23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -892,13 +892,13 @@
         <v>23CopPar</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -910,10 +910,10 @@
         <v>9</v>
       </c>
       <c r="C25" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -922,13 +922,13 @@
         <v>25LigPer</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -937,13 +937,13 @@
         <v>26CopPer</v>
       </c>
       <c r="B27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -952,13 +952,13 @@
         <v>27CopPer</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -967,13 +967,13 @@
         <v>28SupPer</v>
       </c>
       <c r="B29" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -982,13 +982,13 @@
         <v>29PriUru</v>
       </c>
       <c r="B30" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D30" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -997,13 +997,13 @@
         <v>30CopUru</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C31" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D31" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
@@ -1015,10 +1015,10 @@
         <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D32" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
@@ -1027,13 +1027,13 @@
         <v>32LigVen</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D33" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
@@ -1042,13 +1042,13 @@
         <v>33CopVen</v>
       </c>
       <c r="B34" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C34" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D34" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
@@ -1057,13 +1057,13 @@
         <v>34CopVen</v>
       </c>
       <c r="B35" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D35" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
@@ -1072,13 +1072,13 @@
         <v>35CopSud</v>
       </c>
       <c r="B36" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C36" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D36" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
@@ -1087,13 +1087,13 @@
         <v>36CopSud</v>
       </c>
       <c r="B37" t="s">
+        <v>43</v>
+      </c>
+      <c r="C37" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" t="s">
         <v>45</v>
-      </c>
-      <c r="C37" t="s">
-        <v>16</v>
-      </c>
-      <c r="D37" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -1102,13 +1102,13 @@
         <v>37RecSud</v>
       </c>
       <c r="B38" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C38" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D38" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>